<commit_message>
final update for today
</commit_message>
<xml_diff>
--- a/storage/cases.xlsx
+++ b/storage/cases.xlsx
@@ -534,7 +534,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">meena salary </t>
+          <t>dallah</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -649,7 +649,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Waiting Me</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -803,7 +803,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Waiting Me</t>
+          <t>Waiting Me.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">

</xml_diff>

<commit_message>
final update 2026/04/06 20:30
</commit_message>
<xml_diff>
--- a/storage/cases.xlsx
+++ b/storage/cases.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,39 +441,40 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>meena salary</t>
+          <t>meena</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>sooyenieal</t>
+          <t>salary</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Waiting Dep</t>
+          <t>Waiting Me</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>meena salary</t>
+          <t>arthur jobs</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">meena salary </t>
+          <t xml:space="preserve">he need jobs
+</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Waiting Dep</t>
+          <t>Waiting Me.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -485,12 +486,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>meena salary</t>
+          <t xml:space="preserve">vera salary </t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">meena salary </t>
+          <t xml:space="preserve">need to release the vera salary </t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -500,19 +501,19 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>meena salary</t>
+          <t>dallah 2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">meena salary </t>
+          <t>new contract.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -522,19 +523,19 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>meena salary</t>
+          <t>uncle sick</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>dallah</t>
+          <t>sick report</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -544,19 +545,19 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>meena salary</t>
+          <t>meena</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">meena salary </t>
+          <t>nurse exit</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -566,19 +567,19 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>meena salary</t>
+          <t>sooyenieal</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">meena salary </t>
+          <t>sooyenieal</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -588,41 +589,42 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>meena salary</t>
+          <t>rabin poudel</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">meena salary </t>
+          <t>rabin</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Waiting Client</t>
+          <t>Waiting Me</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>meena salary</t>
+          <t>rabin 2</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">meena salary </t>
+          <t xml:space="preserve">rabin 2
+</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -632,397 +634,74 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>meena salary</t>
+          <t>test 2</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">meena salary </t>
+          <t xml:space="preserve">test 2
+</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Waiting Me</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>meena salary</t>
+          <t>test 3</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">meena salary </t>
+          <t>test 3</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Waiting Me.</t>
+          <t>Waiting Dep</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>meena salary</t>
+          <t>orchid</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">meena salary </t>
+          <t>orchid</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Waiting Client</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>meena salary</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">meena salary </t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Waiting Me</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>meena salary</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">meena salary </t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Waiting Me</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>meena salary</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">meena salary </t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Waiting Me</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>meena salary</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">meena salary </t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Waiting Me</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>meena salary</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">meena salary </t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Waiting Me.</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>timesheet of dallah.</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">dallah nammar timesheet is pending. 
-</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Waiting Client</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>timesheet of dallah.</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">dallah nammar timesheet is pending. 
-</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Waiting Client</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>timesheet of dallah.</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">dallah nammar timesheet is pending. 
-</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Waiting Client</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>timesheet of dallah.</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">dallah nammar timesheet is pending. 
-</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Waiting Client</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>timesheet of dallah.</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">dallah nammar timesheet is pending. 
-</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">dallah. </t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">timesheet and exit. </t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Waiting Me</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">orchid </t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>client need to meet mr alshayaa.</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Waiting Me</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Waiting Client</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>my increment.</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">my increment should be done. </t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Waiting Me</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>

</xml_diff>